<commit_message>
commit - working - will add TPS code next
</commit_message>
<xml_diff>
--- a/gemini8048/bin/87KLR951.xlsx
+++ b/gemini8048/bin/87KLR951.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mike/coding_projects/944/DME_sim/gemini8048/bin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C6097D6-962B-2940-8DD9-568913FB064C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EFA0F05-AC71-694D-9A54-DEA9E9F0CFF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12960" yWindow="16720" windowWidth="47100" windowHeight="24480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37360" yWindow="8740" windowWidth="47100" windowHeight="24480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ASM" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8127" uniqueCount="4400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8162" uniqueCount="4429">
   <si>
     <t>https://junctionbyte.com/8051-microcontroller-special-function-registers/</t>
   </si>
@@ -13247,6 +13247,93 @@
   </si>
   <si>
     <t>// END function table adc_map_sensor_read:</t>
+  </si>
+  <si>
+    <t>Long</t>
+  </si>
+  <si>
+    <t>interrupt_info</t>
+  </si>
+  <si>
+    <t>num_timer_ints</t>
+  </si>
+  <si>
+    <t>dec_interrupts</t>
+  </si>
+  <si>
+    <t>timer_period</t>
+  </si>
+  <si>
+    <t>battery_volts</t>
+  </si>
+  <si>
+    <t>knock_raw</t>
+  </si>
+  <si>
+    <t>knock_test_out</t>
+  </si>
+  <si>
+    <t>throttle_degrees</t>
+  </si>
+  <si>
+    <t>throttle_raw_sensor</t>
+  </si>
+  <si>
+    <t>WOT_angle</t>
+  </si>
+  <si>
+    <t>mac_knock_thresh</t>
+  </si>
+  <si>
+    <t>integrated_knock_val</t>
+  </si>
+  <si>
+    <t>knock_det_threshold</t>
+  </si>
+  <si>
+    <t>throttle_position_threshold</t>
+  </si>
+  <si>
+    <t>cycle_count_before_restore</t>
+  </si>
+  <si>
+    <t>max_timing_retart</t>
+  </si>
+  <si>
+    <t>boost_threshold</t>
+  </si>
+  <si>
+    <t>cycle_count_before_pulling_boost</t>
+  </si>
+  <si>
+    <t>cycle_count_before_restore_boost</t>
+  </si>
+  <si>
+    <t>TPS Voltage</t>
+  </si>
+  <si>
+    <t>TPS_Cycling</t>
+  </si>
+  <si>
+    <t>TPS_Scaling</t>
+  </si>
+  <si>
+    <t>//3bh - The scaling numerator 3B is initialized to 119 in the trigger/reset routine. So the nominal scaling factor is 119/256, or about 0.46</t>
+  </si>
+  <si>
+    <t>//value ranging from 0-27, used for cycling value control map lookups</t>
+  </si>
+  <si>
+    <t>throt_pos_thresh</t>
+  </si>
+  <si>
+    <t>boost_thresh</t>
+  </si>
+  <si>
+    <t>knk_thres_cyl</t>
+  </si>
+  <si>
+    <t>knock_thresh_coeef</t>
   </si>
 </sst>
 </file>
@@ -13350,7 +13437,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -13409,6 +13496,7 @@
     <xf numFmtId="6" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -40158,1267 +40246,1470 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K129"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="22"/>
   <cols>
     <col min="1" max="1" width="35.6640625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="37.83203125" style="12" customWidth="1"/>
-    <col min="3" max="3" width="98.6640625" style="15" customWidth="1"/>
-    <col min="4" max="4" width="39.33203125" style="17" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="9" customWidth="1"/>
-    <col min="6" max="16384" width="10.83203125" style="9"/>
+    <col min="2" max="3" width="37.83203125" style="12" customWidth="1"/>
+    <col min="4" max="4" width="98.6640625" style="15" customWidth="1"/>
+    <col min="5" max="5" width="39.33203125" style="17" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" style="9" customWidth="1"/>
+    <col min="7" max="16384" width="10.83203125" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="23" customHeight="1">
+    <row r="1" spans="1:11" ht="23" customHeight="1">
       <c r="A1" s="8" t="s">
         <v>3787</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>3788</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="11" t="s">
         <v>3789</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="14" t="s">
+        <v>4400</v>
+      </c>
+      <c r="E1" s="17" t="s">
         <v>3790</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="46" customHeight="1">
+    <row r="2" spans="1:11" ht="46" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>3791</v>
       </c>
       <c r="B2" s="12">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="9" t="s">
+        <v>4401</v>
+      </c>
+      <c r="D2" s="15" t="s">
         <v>3792</v>
       </c>
-      <c r="D2" s="18">
+      <c r="E2" s="18">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:11">
       <c r="B3" s="12">
         <v>1</v>
       </c>
-      <c r="D3" s="18">
+      <c r="C3" s="9"/>
+      <c r="E3" s="18">
         <v>23</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>3793</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="23" customHeight="1">
+    <row r="4" spans="1:11" ht="23" customHeight="1">
       <c r="A4" s="9" t="s">
         <v>3794</v>
       </c>
       <c r="B4" s="12">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="9" t="s">
+        <v>4402</v>
+      </c>
+      <c r="D4" s="15" t="s">
         <v>3795</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="E4" s="18" t="s">
         <v>3796</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="23" customHeight="1">
+    <row r="5" spans="1:11" ht="23" customHeight="1">
       <c r="A5" s="9" t="s">
         <v>3797</v>
       </c>
       <c r="B5" s="12">
         <v>3</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="9" t="s">
+        <v>3797</v>
+      </c>
+      <c r="D5" s="15" t="s">
         <v>3798</v>
       </c>
-      <c r="D5" s="18">
+      <c r="E5" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:11">
       <c r="B6" s="12">
         <v>4</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="C6" s="9"/>
+      <c r="E6" s="18" t="s">
         <v>3799</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="23" customHeight="1">
+    <row r="7" spans="1:11" ht="23" customHeight="1">
       <c r="A7" s="9" t="s">
         <v>3800</v>
       </c>
       <c r="B7" s="12">
         <v>5</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="9" t="s">
+        <v>4403</v>
+      </c>
+      <c r="D7" s="15" t="s">
         <v>3801</v>
       </c>
-      <c r="D7" s="18">
+      <c r="E7" s="18">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="46" customHeight="1">
+    <row r="8" spans="1:11" ht="46" customHeight="1">
       <c r="A8" s="9" t="s">
         <v>3802</v>
       </c>
       <c r="B8" s="12">
         <v>6</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="9" t="s">
+        <v>3802</v>
+      </c>
+      <c r="D8" s="15" t="s">
         <v>3803</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>3804</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="92" customHeight="1">
+    <row r="9" spans="1:11" ht="92" customHeight="1">
       <c r="A9" s="9" t="s">
         <v>3805</v>
       </c>
       <c r="B9" s="12">
         <v>7</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="9" t="s">
+        <v>4404</v>
+      </c>
+      <c r="D9" s="15" t="s">
         <v>3806</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="E9" s="18" t="s">
         <v>1586</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:11">
       <c r="B10" s="12">
         <v>8</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="C10" s="9"/>
+      <c r="E10" s="18" t="s">
         <v>3807</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:11">
       <c r="B11" s="12">
         <v>9</v>
       </c>
-      <c r="D11" s="18">
+      <c r="C11" s="9"/>
+      <c r="E11" s="18">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:11">
       <c r="B12" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="C12" s="9"/>
+      <c r="E12" s="18" t="s">
         <v>3808</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:11">
       <c r="B13" s="12" t="s">
         <v>3809</v>
       </c>
-      <c r="D13" s="18">
+      <c r="C13" s="9"/>
+      <c r="E13" s="18">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:11">
       <c r="B14" s="12" t="s">
         <v>529</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="C14" s="9"/>
+      <c r="E14" s="18" t="s">
         <v>3810</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:11">
       <c r="B15" s="12" t="s">
         <v>3811</v>
       </c>
-      <c r="D15" s="18">
+      <c r="C15" s="9"/>
+      <c r="E15" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:11">
       <c r="B16" s="12" t="s">
         <v>3812</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="C16" s="9"/>
+      <c r="E16" s="18" t="s">
         <v>3807</v>
       </c>
     </row>
-    <row r="17" spans="2:4">
+    <row r="17" spans="2:5">
       <c r="B17" s="12" t="s">
         <v>3813</v>
       </c>
-      <c r="D17" s="18">
+      <c r="C17" s="9"/>
+      <c r="E17" s="18">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="23" customHeight="1">
+    <row r="18" spans="2:5" ht="23" customHeight="1">
       <c r="B18" s="12">
         <v>10</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="9"/>
+      <c r="D18" s="15" t="s">
         <v>3814</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="E18" s="18" t="s">
         <v>3808</v>
       </c>
     </row>
-    <row r="19" spans="2:4">
+    <row r="19" spans="2:5">
       <c r="B19" s="12">
         <v>11</v>
       </c>
-      <c r="D19" s="18">
+      <c r="C19" s="9"/>
+      <c r="E19" s="18">
         <v>81</v>
       </c>
     </row>
-    <row r="20" spans="2:4">
+    <row r="20" spans="2:5">
       <c r="B20" s="12">
         <v>12</v>
       </c>
-      <c r="D20" s="18">
+      <c r="C20" s="9"/>
+      <c r="E20" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:4">
+    <row r="21" spans="2:5">
       <c r="B21" s="12">
         <v>13</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="C21" s="9"/>
+      <c r="E21" s="18" t="s">
         <v>3815</v>
       </c>
     </row>
-    <row r="22" spans="2:4">
+    <row r="22" spans="2:5">
       <c r="B22" s="12">
         <v>14</v>
       </c>
-      <c r="D22" s="18">
+      <c r="C22" s="9"/>
+      <c r="E22" s="18">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="2:4">
+    <row r="23" spans="2:5">
       <c r="B23" s="12">
         <v>15</v>
       </c>
-      <c r="D23" s="18">
+      <c r="C23" s="9"/>
+      <c r="E23" s="18">
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="2:4">
+    <row r="24" spans="2:5">
       <c r="B24" s="12">
         <v>16</v>
       </c>
-      <c r="D24" s="18">
+      <c r="C24" s="9"/>
+      <c r="E24" s="18">
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="2:4">
+    <row r="25" spans="2:5">
       <c r="B25" s="12">
         <v>17</v>
       </c>
-      <c r="D25" s="18">
+      <c r="C25" s="9"/>
+      <c r="E25" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:4">
+    <row r="26" spans="2:5">
       <c r="B26" s="12">
         <v>18</v>
       </c>
-      <c r="D26" s="18">
+      <c r="C26" s="9"/>
+      <c r="E26" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:4">
+    <row r="27" spans="2:5">
       <c r="B27" s="12">
         <v>19</v>
       </c>
-      <c r="D27" s="18">
+      <c r="C27" s="9"/>
+      <c r="E27" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:4">
+    <row r="28" spans="2:5">
       <c r="B28" s="12" t="s">
         <v>3816</v>
       </c>
-      <c r="D28" s="18">
+      <c r="C28" s="9"/>
+      <c r="E28" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:4">
+    <row r="29" spans="2:5">
       <c r="B29" s="12" t="s">
         <v>3817</v>
       </c>
-      <c r="D29" s="18">
+      <c r="C29" s="9"/>
+      <c r="E29" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:4">
+    <row r="30" spans="2:5">
       <c r="B30" s="12" t="s">
         <v>3818</v>
       </c>
-      <c r="D30" s="18">
+      <c r="C30" s="9"/>
+      <c r="E30" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:4">
+    <row r="31" spans="2:5">
       <c r="B31" s="12" t="s">
         <v>3819</v>
       </c>
-      <c r="D31" s="18">
+      <c r="C31" s="9"/>
+      <c r="E31" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:4">
+    <row r="32" spans="2:5">
       <c r="B32" s="12" t="s">
         <v>3820</v>
       </c>
-      <c r="D32" s="18">
+      <c r="C32" s="9"/>
+      <c r="E32" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:12">
       <c r="B33" s="12" t="s">
         <v>3821</v>
       </c>
-      <c r="D33" s="18">
+      <c r="C33" s="9"/>
+      <c r="E33" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:12">
       <c r="B34" s="12">
         <v>20</v>
       </c>
-      <c r="D34" s="18">
+      <c r="C34" s="9"/>
+      <c r="E34" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" spans="1:12">
       <c r="B35" s="12">
         <v>21</v>
       </c>
-      <c r="D35" s="18">
+      <c r="C35" s="9"/>
+      <c r="E35" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:11">
+    <row r="36" spans="1:12">
       <c r="B36" s="12">
         <v>22</v>
       </c>
-      <c r="D36" s="18" t="s">
+      <c r="C36" s="9"/>
+      <c r="E36" s="18" t="s">
         <v>3804</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" spans="1:12">
       <c r="B37" s="12">
         <v>23</v>
       </c>
-      <c r="D37" s="18">
+      <c r="C37" s="9"/>
+      <c r="E37" s="18">
         <v>2</v>
       </c>
-      <c r="J37" s="10"/>
-    </row>
-    <row r="38" spans="1:11" ht="23" customHeight="1">
+      <c r="K37" s="10"/>
+    </row>
+    <row r="38" spans="1:12" ht="23" customHeight="1">
       <c r="A38" s="9" t="s">
         <v>3822</v>
       </c>
       <c r="B38" s="12">
         <v>24</v>
       </c>
-      <c r="C38" s="15" t="s">
+      <c r="C38" s="9" t="s">
+        <v>3822</v>
+      </c>
+      <c r="D38" s="15" t="s">
         <v>3823</v>
       </c>
-      <c r="D38" s="18" t="s">
+      <c r="E38" s="18" t="s">
         <v>3824</v>
       </c>
-      <c r="J38" s="10"/>
-    </row>
-    <row r="39" spans="1:11">
+      <c r="K38" s="10"/>
+    </row>
+    <row r="39" spans="1:12">
       <c r="B39" s="12">
         <v>25</v>
       </c>
-      <c r="D39" s="18">
+      <c r="C39" s="9"/>
+      <c r="E39" s="18">
         <v>0</v>
       </c>
-      <c r="J39" s="10"/>
-    </row>
-    <row r="40" spans="1:11">
+      <c r="K39" s="10"/>
+    </row>
+    <row r="40" spans="1:12">
       <c r="B40" s="12">
         <v>26</v>
       </c>
-      <c r="D40" s="18">
+      <c r="C40" s="9"/>
+      <c r="E40" s="18">
         <v>0</v>
       </c>
-      <c r="J40" s="10"/>
-    </row>
-    <row r="41" spans="1:11">
+      <c r="K40" s="10"/>
+    </row>
+    <row r="41" spans="1:12">
       <c r="B41" s="12">
         <v>27</v>
       </c>
-      <c r="D41" s="18">
+      <c r="C41" s="9"/>
+      <c r="E41" s="18">
         <v>27</v>
       </c>
-      <c r="J41" s="10"/>
-    </row>
-    <row r="42" spans="1:11">
+      <c r="K41" s="10"/>
+    </row>
+    <row r="42" spans="1:12">
       <c r="B42" s="12">
         <v>28</v>
       </c>
-      <c r="D42" s="18">
+      <c r="C42" s="9"/>
+      <c r="E42" s="18">
         <v>0</v>
       </c>
-      <c r="J42" s="10"/>
-    </row>
-    <row r="43" spans="1:11">
+      <c r="K42" s="10"/>
+    </row>
+    <row r="43" spans="1:12">
       <c r="B43" s="12">
         <v>29</v>
       </c>
-      <c r="D43" s="18">
+      <c r="C43" s="9"/>
+      <c r="E43" s="18">
         <v>0</v>
       </c>
-      <c r="K43" s="10"/>
-    </row>
-    <row r="44" spans="1:11" ht="45" customHeight="1">
+      <c r="L43" s="10"/>
+    </row>
+    <row r="44" spans="1:12" ht="45" customHeight="1">
       <c r="B44" s="13" t="s">
         <v>3825</v>
       </c>
-      <c r="C44" s="16" t="s">
+      <c r="C44" s="9"/>
+      <c r="D44" s="16" t="s">
         <v>3826</v>
       </c>
-      <c r="D44" s="18" t="s">
+      <c r="E44" s="18" t="s">
         <v>3827</v>
       </c>
-      <c r="K44" s="10"/>
-    </row>
-    <row r="45" spans="1:11" ht="23" customHeight="1">
+      <c r="L44" s="10"/>
+    </row>
+    <row r="45" spans="1:12" ht="23" customHeight="1">
       <c r="B45" s="13" t="s">
         <v>3828</v>
       </c>
-      <c r="C45" s="16" t="s">
+      <c r="C45" s="9"/>
+      <c r="D45" s="16" t="s">
         <v>3829</v>
       </c>
-      <c r="D45" s="18" t="s">
+      <c r="E45" s="18" t="s">
         <v>3817</v>
       </c>
-      <c r="J45" s="10"/>
-    </row>
-    <row r="46" spans="1:11">
+      <c r="K45" s="10"/>
+    </row>
+    <row r="46" spans="1:12">
       <c r="B46" s="12" t="s">
         <v>3830</v>
       </c>
-      <c r="D46" s="18">
+      <c r="C46" s="9"/>
+      <c r="E46" s="18">
         <v>0</v>
       </c>
-      <c r="J46" s="10"/>
-    </row>
-    <row r="47" spans="1:11">
+      <c r="K46" s="10"/>
+    </row>
+    <row r="47" spans="1:12">
       <c r="B47" s="12" t="s">
         <v>3831</v>
       </c>
-      <c r="D47" s="18">
+      <c r="C47" s="9"/>
+      <c r="E47" s="18">
         <v>0</v>
       </c>
-      <c r="J47" s="10"/>
-    </row>
-    <row r="48" spans="1:11">
+      <c r="K47" s="10"/>
+    </row>
+    <row r="48" spans="1:12">
       <c r="A48" s="9" t="s">
         <v>3832</v>
       </c>
       <c r="B48" s="12" t="s">
         <v>3833</v>
       </c>
-      <c r="D48" s="18" t="s">
+      <c r="C48" s="9" t="s">
+        <v>4405</v>
+      </c>
+      <c r="E48" s="18" t="s">
         <v>3834</v>
       </c>
-      <c r="J48" s="10"/>
-    </row>
-    <row r="49" spans="1:10" ht="23" customHeight="1">
+      <c r="K48" s="10"/>
+    </row>
+    <row r="49" spans="1:11" ht="23" customHeight="1">
       <c r="A49" s="9" t="s">
         <v>3835</v>
       </c>
       <c r="B49" s="12" t="s">
         <v>3836</v>
       </c>
-      <c r="C49" s="15" t="s">
+      <c r="C49" s="9" t="s">
+        <v>4406</v>
+      </c>
+      <c r="D49" s="15" t="s">
         <v>3837</v>
       </c>
-      <c r="D49" s="18">
+      <c r="E49" s="18">
         <v>0</v>
       </c>
-      <c r="J49" s="10"/>
-    </row>
-    <row r="50" spans="1:10">
+      <c r="K49" s="10"/>
+    </row>
+    <row r="50" spans="1:11">
       <c r="B50" s="12">
         <v>30</v>
       </c>
-      <c r="D50" s="18" t="s">
+      <c r="C50" s="9"/>
+      <c r="E50" s="18" t="s">
         <v>3834</v>
       </c>
-      <c r="J50" s="10"/>
-    </row>
-    <row r="51" spans="1:10">
+      <c r="K50" s="10"/>
+    </row>
+    <row r="51" spans="1:11">
       <c r="A51" s="9" t="s">
         <v>3838</v>
       </c>
       <c r="B51" s="12">
         <v>31</v>
       </c>
-      <c r="D51" s="18">
+      <c r="C51" s="9" t="s">
+        <v>4407</v>
+      </c>
+      <c r="E51" s="18">
         <v>0</v>
       </c>
-      <c r="J51" s="10"/>
-    </row>
-    <row r="52" spans="1:10">
+      <c r="K51" s="10"/>
+    </row>
+    <row r="52" spans="1:11">
       <c r="B52" s="12">
         <v>32</v>
       </c>
-      <c r="D52" s="18">
+      <c r="C52" s="9"/>
+      <c r="E52" s="18">
         <v>0</v>
       </c>
-      <c r="J52" s="10"/>
-    </row>
-    <row r="53" spans="1:10" ht="23" customHeight="1">
+      <c r="K52" s="10"/>
+    </row>
+    <row r="53" spans="1:11" ht="23" customHeight="1">
       <c r="A53" s="9" t="s">
         <v>3839</v>
       </c>
       <c r="B53" s="12">
         <v>33</v>
       </c>
-      <c r="C53" s="15" t="s">
+      <c r="C53" s="9" t="s">
+        <v>3839</v>
+      </c>
+      <c r="D53" s="15" t="s">
         <v>3840</v>
       </c>
-      <c r="D53" s="18">
+      <c r="E53" s="18">
         <v>0</v>
       </c>
-      <c r="J53" s="10"/>
-    </row>
-    <row r="54" spans="1:10">
+      <c r="K53" s="10"/>
+    </row>
+    <row r="54" spans="1:11">
       <c r="B54" s="12">
         <v>34</v>
       </c>
-      <c r="D54" s="18">
+      <c r="C54" s="9"/>
+      <c r="E54" s="18">
         <v>6</v>
       </c>
-      <c r="J54" s="10"/>
-    </row>
-    <row r="55" spans="1:10">
+      <c r="K54" s="10"/>
+    </row>
+    <row r="55" spans="1:11">
       <c r="B55" s="12">
         <v>35</v>
       </c>
-      <c r="D55" s="18" t="s">
+      <c r="C55" s="9"/>
+      <c r="E55" s="18" t="s">
         <v>3834</v>
       </c>
-      <c r="J55" s="10"/>
-    </row>
-    <row r="56" spans="1:10">
+      <c r="K55" s="10"/>
+    </row>
+    <row r="56" spans="1:11">
       <c r="B56" s="12">
         <v>36</v>
       </c>
-      <c r="D56" s="18" t="s">
+      <c r="C56" s="9"/>
+      <c r="E56" s="18" t="s">
         <v>3834</v>
       </c>
-      <c r="J56" s="10"/>
-    </row>
-    <row r="57" spans="1:10">
+      <c r="K56" s="10"/>
+    </row>
+    <row r="57" spans="1:11">
       <c r="B57" s="12">
         <v>37</v>
       </c>
-      <c r="D57" s="18">
+      <c r="C57" s="9"/>
+      <c r="E57" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="46" customHeight="1">
+    <row r="58" spans="1:11" ht="46" customHeight="1">
       <c r="A58" s="9" t="s">
         <v>3841</v>
       </c>
       <c r="B58" s="12">
         <v>38</v>
       </c>
-      <c r="C58" s="15" t="s">
+      <c r="C58" s="9" t="s">
+        <v>3841</v>
+      </c>
+      <c r="D58" s="15" t="s">
         <v>3842</v>
       </c>
-      <c r="D58" s="18">
+      <c r="E58" s="18">
         <v>71</v>
       </c>
-      <c r="J58" s="10"/>
-    </row>
-    <row r="59" spans="1:10" ht="23" customHeight="1">
+      <c r="K58" s="10"/>
+    </row>
+    <row r="59" spans="1:11" ht="23" customHeight="1">
       <c r="A59" s="9" t="s">
         <v>3843</v>
       </c>
       <c r="B59" s="12">
         <v>39</v>
       </c>
-      <c r="C59" s="15" t="s">
+      <c r="C59" s="9" t="s">
+        <v>4420</v>
+      </c>
+      <c r="D59" s="15" t="s">
         <v>3844</v>
       </c>
-      <c r="D59" s="18" t="s">
+      <c r="E59" s="18" t="s">
         <v>3845</v>
       </c>
-      <c r="J59" s="10"/>
-    </row>
-    <row r="60" spans="1:10" ht="23" customHeight="1">
+      <c r="K59" s="10"/>
+    </row>
+    <row r="60" spans="1:11" ht="23" customHeight="1">
       <c r="A60" s="9" t="s">
         <v>3846</v>
       </c>
       <c r="B60" s="12" t="s">
         <v>3847</v>
       </c>
-      <c r="C60" s="15" t="s">
+      <c r="C60" s="9" t="s">
+        <v>4408</v>
+      </c>
+      <c r="D60" s="15" t="s">
         <v>3848</v>
       </c>
-      <c r="D60" s="18">
+      <c r="E60" s="18">
         <v>0</v>
       </c>
-      <c r="J60" s="10"/>
-    </row>
-    <row r="61" spans="1:10">
+      <c r="K60" s="10"/>
+    </row>
+    <row r="61" spans="1:11" ht="46">
       <c r="B61" s="12" t="s">
         <v>3849</v>
       </c>
-      <c r="D61" s="18">
+      <c r="C61" s="9" t="s">
+        <v>4422</v>
+      </c>
+      <c r="D61" s="15" t="s">
+        <v>4423</v>
+      </c>
+      <c r="E61" s="18">
         <v>77</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="23" customHeight="1">
+    <row r="62" spans="1:11" ht="23" customHeight="1">
       <c r="A62" s="9" t="s">
         <v>3850</v>
       </c>
       <c r="B62" s="12" t="s">
         <v>3851</v>
       </c>
-      <c r="C62" s="15" t="s">
+      <c r="C62" s="9" t="s">
+        <v>4409</v>
+      </c>
+      <c r="D62" s="15" t="s">
         <v>3852</v>
       </c>
-      <c r="D62" s="18">
+      <c r="E62" s="18">
         <v>77</v>
       </c>
-      <c r="J62" s="10"/>
-    </row>
-    <row r="63" spans="1:10">
+      <c r="K62" s="10"/>
+    </row>
+    <row r="63" spans="1:11">
       <c r="B63" s="12" t="s">
         <v>3853</v>
       </c>
-      <c r="D63" s="18">
+      <c r="C63" s="9"/>
+      <c r="E63" s="18">
         <v>77</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="23" customHeight="1">
+    <row r="64" spans="1:11" ht="23" customHeight="1">
       <c r="B64" s="13" t="s">
         <v>3854</v>
       </c>
-      <c r="C64" s="16" t="s">
+      <c r="C64" s="9" t="s">
+        <v>4410</v>
+      </c>
+      <c r="D64" s="16" t="s">
         <v>3855</v>
       </c>
-      <c r="D64" s="18">
+      <c r="E64" s="18">
         <v>77</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:11">
       <c r="B65" s="12" t="s">
         <v>3856</v>
       </c>
-      <c r="D65" s="18">
+      <c r="C65" s="9"/>
+      <c r="E65" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
+    <row r="66" spans="1:11">
       <c r="B66" s="12">
         <v>40</v>
       </c>
-      <c r="D66" s="18">
+      <c r="C66" s="9"/>
+      <c r="E66" s="18">
         <v>77</v>
       </c>
     </row>
-    <row r="67" spans="1:10">
+    <row r="67" spans="1:11">
       <c r="B67" s="12">
         <v>41</v>
       </c>
-      <c r="D67" s="18">
+      <c r="C67" s="9"/>
+      <c r="E67" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:10">
+    <row r="68" spans="1:11">
       <c r="B68" s="12">
         <v>42</v>
       </c>
-      <c r="D68" s="18">
+      <c r="C68" s="9"/>
+      <c r="E68" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:10">
+    <row r="69" spans="1:11">
       <c r="B69" s="12">
         <v>43</v>
       </c>
-      <c r="D69" s="18">
+      <c r="C69" s="9" t="s">
+        <v>4421</v>
+      </c>
+      <c r="D69" s="26" t="s">
+        <v>4424</v>
+      </c>
+      <c r="E69" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="23" customHeight="1">
+    <row r="70" spans="1:11" ht="23" customHeight="1">
       <c r="A70" s="9" t="s">
         <v>3857</v>
       </c>
       <c r="B70" s="12">
         <v>44</v>
       </c>
-      <c r="C70" s="15" t="s">
+      <c r="C70" s="9" t="s">
+        <v>3857</v>
+      </c>
+      <c r="D70" s="15" t="s">
         <v>3858</v>
       </c>
-      <c r="D70" s="18">
+      <c r="E70" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="69" customHeight="1">
+    <row r="71" spans="1:11" ht="69" customHeight="1">
       <c r="A71" s="9" t="s">
         <v>3859</v>
       </c>
       <c r="B71" s="12">
         <v>45</v>
       </c>
-      <c r="C71" s="15" t="s">
+      <c r="C71" s="9" t="s">
+        <v>4411</v>
+      </c>
+      <c r="D71" s="15" t="s">
         <v>3860</v>
       </c>
-      <c r="D71" s="18">
+      <c r="E71" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="23" customHeight="1">
+    <row r="72" spans="1:11" ht="23" customHeight="1">
       <c r="A72" s="9" t="s">
         <v>3861</v>
       </c>
       <c r="B72" s="12">
         <v>46</v>
       </c>
-      <c r="C72" s="15" t="s">
+      <c r="C72" s="9" t="s">
+        <v>4412</v>
+      </c>
+      <c r="D72" s="15" t="s">
         <v>3862</v>
       </c>
-      <c r="D72" s="18">
+      <c r="E72" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="45" customHeight="1">
+    <row r="73" spans="1:11" ht="45" customHeight="1">
+      <c r="A73" s="9" t="s">
+        <v>4428</v>
+      </c>
       <c r="B73" s="13">
         <v>47</v>
       </c>
-      <c r="C73" s="16" t="s">
+      <c r="C73" s="9" t="s">
+        <v>4413</v>
+      </c>
+      <c r="D73" s="16" t="s">
         <v>3863</v>
       </c>
-      <c r="D73" s="18">
+      <c r="E73" s="18">
         <v>0</v>
       </c>
-      <c r="J73" s="10"/>
-    </row>
-    <row r="74" spans="1:10" ht="23" customHeight="1">
+      <c r="K73" s="10"/>
+    </row>
+    <row r="74" spans="1:11" ht="23" customHeight="1">
+      <c r="A74" s="9" t="s">
+        <v>4425</v>
+      </c>
       <c r="B74" s="13">
         <v>48</v>
       </c>
-      <c r="C74" s="16" t="s">
+      <c r="C74" s="9" t="s">
+        <v>4414</v>
+      </c>
+      <c r="D74" s="16" t="s">
         <v>3864</v>
       </c>
-      <c r="D74" s="18">
+      <c r="E74" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:10">
+    <row r="75" spans="1:11">
       <c r="B75" s="13">
         <v>49</v>
       </c>
-      <c r="C75" s="16"/>
-      <c r="D75" s="18">
+      <c r="C75" s="9"/>
+      <c r="D75" s="16"/>
+      <c r="E75" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="45" customHeight="1">
+    <row r="76" spans="1:11" ht="45" customHeight="1">
       <c r="B76" s="13" t="s">
         <v>3865</v>
       </c>
-      <c r="C76" s="16" t="s">
+      <c r="C76" s="9" t="s">
+        <v>4415</v>
+      </c>
+      <c r="D76" s="16" t="s">
         <v>3866</v>
       </c>
-      <c r="D76" s="18">
+      <c r="E76" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="45" customHeight="1">
+    <row r="77" spans="1:11" ht="45" customHeight="1">
       <c r="B77" s="13" t="s">
         <v>3867</v>
       </c>
-      <c r="C77" s="16" t="s">
+      <c r="C77" s="9" t="s">
+        <v>4416</v>
+      </c>
+      <c r="D77" s="16" t="s">
         <v>3868</v>
       </c>
-      <c r="D77" s="18">
+      <c r="E77" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="23" customHeight="1">
+    <row r="78" spans="1:11" ht="23" customHeight="1">
+      <c r="A78" s="9" t="s">
+        <v>4426</v>
+      </c>
       <c r="B78" s="13" t="s">
         <v>3869</v>
       </c>
-      <c r="C78" s="16" t="s">
+      <c r="C78" s="9" t="s">
+        <v>4417</v>
+      </c>
+      <c r="D78" s="16" t="s">
         <v>3870</v>
       </c>
-      <c r="D78" s="18">
+      <c r="E78" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:10">
+    <row r="79" spans="1:11">
       <c r="B79" s="13" t="s">
         <v>3871</v>
       </c>
-      <c r="C79" s="16"/>
-      <c r="D79" s="18">
+      <c r="C79" s="9"/>
+      <c r="D79" s="16"/>
+      <c r="E79" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="23" customHeight="1">
+    <row r="80" spans="1:11" ht="23" customHeight="1">
       <c r="B80" s="13" t="s">
         <v>3872</v>
       </c>
-      <c r="C80" s="16" t="s">
+      <c r="C80" s="9" t="s">
+        <v>4418</v>
+      </c>
+      <c r="D80" s="16" t="s">
         <v>3873</v>
       </c>
-      <c r="D80" s="18">
+      <c r="E80" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="2:4">
+    <row r="81" spans="2:5">
       <c r="B81" s="13" t="s">
         <v>3874</v>
       </c>
-      <c r="C81" s="16"/>
-      <c r="D81" s="18">
+      <c r="C81" s="9"/>
+      <c r="D81" s="16"/>
+      <c r="E81" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="2:4" ht="23" customHeight="1">
+    <row r="82" spans="2:5" ht="23" customHeight="1">
       <c r="B82" s="13">
         <v>50</v>
       </c>
-      <c r="C82" s="16" t="s">
+      <c r="C82" s="9" t="s">
+        <v>4419</v>
+      </c>
+      <c r="D82" s="16" t="s">
         <v>3875</v>
       </c>
-      <c r="D82" s="18">
+      <c r="E82" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="2:4">
+    <row r="83" spans="2:5">
       <c r="B83" s="13">
         <v>51</v>
       </c>
-      <c r="C83" s="16"/>
-      <c r="D83" s="18">
+      <c r="C83" s="9"/>
+      <c r="D83" s="16"/>
+      <c r="E83" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="2:4">
+    <row r="84" spans="2:5">
       <c r="B84" s="13">
         <v>52</v>
       </c>
-      <c r="C84" s="16"/>
-      <c r="D84" s="18">
+      <c r="C84" s="9"/>
+      <c r="D84" s="16"/>
+      <c r="E84" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="2:4">
+    <row r="85" spans="2:5">
       <c r="B85" s="13">
         <v>53</v>
       </c>
-      <c r="C85" s="16"/>
-      <c r="D85" s="18">
+      <c r="C85" s="9"/>
+      <c r="D85" s="16"/>
+      <c r="E85" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="2:4">
+    <row r="86" spans="2:5">
       <c r="B86" s="13">
         <v>54</v>
       </c>
-      <c r="C86" s="16"/>
-      <c r="D86" s="18">
+      <c r="C86" s="9"/>
+      <c r="D86" s="16"/>
+      <c r="E86" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="2:4">
+    <row r="87" spans="2:5">
       <c r="B87" s="13">
         <v>55</v>
       </c>
-      <c r="C87" s="16"/>
-      <c r="D87" s="18">
+      <c r="C87" s="9"/>
+      <c r="D87" s="16"/>
+      <c r="E87" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="2:4">
+    <row r="88" spans="2:5">
       <c r="B88" s="13">
         <v>56</v>
       </c>
-      <c r="C88" s="16"/>
-      <c r="D88" s="18">
+      <c r="C88" s="9"/>
+      <c r="D88" s="16"/>
+      <c r="E88" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="2:4">
+    <row r="89" spans="2:5">
       <c r="B89" s="13">
         <v>57</v>
       </c>
-      <c r="C89" s="16"/>
-      <c r="D89" s="18">
+      <c r="C89" s="9"/>
+      <c r="D89" s="16"/>
+      <c r="E89" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="2:4">
+    <row r="90" spans="2:5">
       <c r="B90" s="13">
         <v>58</v>
       </c>
-      <c r="C90" s="16"/>
-      <c r="D90" s="18">
+      <c r="C90" s="9"/>
+      <c r="D90" s="16"/>
+      <c r="E90" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="2:4">
+    <row r="91" spans="2:5">
       <c r="B91" s="13">
         <v>59</v>
       </c>
-      <c r="C91" s="16"/>
-      <c r="D91" s="18">
+      <c r="C91" s="9"/>
+      <c r="D91" s="16"/>
+      <c r="E91" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="2:4">
+    <row r="92" spans="2:5">
       <c r="B92" s="13" t="s">
         <v>3876</v>
       </c>
-      <c r="C92" s="16"/>
-      <c r="D92" s="18">
+      <c r="C92" s="9"/>
+      <c r="D92" s="16"/>
+      <c r="E92" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="2:4">
+    <row r="93" spans="2:5">
       <c r="B93" s="13" t="s">
         <v>3877</v>
       </c>
-      <c r="C93" s="16"/>
-      <c r="D93" s="18">
+      <c r="C93" s="9"/>
+      <c r="D93" s="16"/>
+      <c r="E93" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="2:4">
+    <row r="94" spans="2:5">
       <c r="B94" s="13" t="s">
         <v>3878</v>
       </c>
-      <c r="C94" s="16"/>
-      <c r="D94" s="18">
+      <c r="C94" s="9"/>
+      <c r="D94" s="16"/>
+      <c r="E94" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="2:4">
+    <row r="95" spans="2:5">
       <c r="B95" s="13" t="s">
         <v>3879</v>
       </c>
-      <c r="C95" s="16"/>
-      <c r="D95" s="18">
+      <c r="C95" s="9"/>
+      <c r="D95" s="16"/>
+      <c r="E95" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="2:4">
+    <row r="96" spans="2:5">
       <c r="B96" s="13" t="s">
         <v>3880</v>
       </c>
-      <c r="C96" s="16"/>
-      <c r="D96" s="18">
+      <c r="C96" s="9"/>
+      <c r="D96" s="16"/>
+      <c r="E96" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="2:4">
+    <row r="97" spans="2:5">
       <c r="B97" s="13" t="s">
         <v>3881</v>
       </c>
-      <c r="C97" s="16"/>
-      <c r="D97" s="18">
+      <c r="C97" s="9"/>
+      <c r="D97" s="16"/>
+      <c r="E97" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="2:4">
+    <row r="98" spans="2:5">
       <c r="B98" s="13">
         <v>60</v>
       </c>
-      <c r="C98" s="16"/>
-      <c r="D98" s="18">
+      <c r="C98" s="9"/>
+      <c r="D98" s="16"/>
+      <c r="E98" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="2:4">
+    <row r="99" spans="2:5">
       <c r="B99" s="13">
         <v>61</v>
       </c>
-      <c r="C99" s="16"/>
-      <c r="D99" s="18">
+      <c r="C99" s="9"/>
+      <c r="D99" s="16"/>
+      <c r="E99" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="2:4">
+    <row r="100" spans="2:5">
       <c r="B100" s="13">
         <v>62</v>
       </c>
-      <c r="C100" s="16"/>
-      <c r="D100" s="18">
+      <c r="C100" s="9"/>
+      <c r="D100" s="16"/>
+      <c r="E100" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="2:4">
+    <row r="101" spans="2:5">
       <c r="B101" s="13">
         <v>63</v>
       </c>
-      <c r="C101" s="16"/>
-      <c r="D101" s="18">
+      <c r="C101" s="9"/>
+      <c r="D101" s="16"/>
+      <c r="E101" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="2:4">
+    <row r="102" spans="2:5">
       <c r="B102" s="13">
         <v>64</v>
       </c>
-      <c r="C102" s="16"/>
-      <c r="D102" s="18">
+      <c r="C102" s="9"/>
+      <c r="D102" s="16"/>
+      <c r="E102" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="2:4">
+    <row r="103" spans="2:5">
       <c r="B103" s="13">
         <v>65</v>
       </c>
-      <c r="C103" s="16"/>
-      <c r="D103" s="18">
+      <c r="C103" s="9"/>
+      <c r="D103" s="16"/>
+      <c r="E103" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="2:4">
+    <row r="104" spans="2:5">
       <c r="B104" s="13">
         <v>66</v>
       </c>
-      <c r="C104" s="16"/>
-      <c r="D104" s="18">
+      <c r="C104" s="9"/>
+      <c r="D104" s="16"/>
+      <c r="E104" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="2:4">
+    <row r="105" spans="2:5">
       <c r="B105" s="13">
         <v>67</v>
       </c>
-      <c r="C105" s="16"/>
-      <c r="D105" s="18">
+      <c r="C105" s="9"/>
+      <c r="D105" s="16"/>
+      <c r="E105" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="2:4">
+    <row r="106" spans="2:5">
       <c r="B106" s="13">
         <v>68</v>
       </c>
-      <c r="C106" s="16"/>
-      <c r="D106" s="18">
+      <c r="C106" s="9"/>
+      <c r="D106" s="16"/>
+      <c r="E106" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="2:4" ht="23" customHeight="1">
+    <row r="107" spans="2:5" ht="23" customHeight="1">
       <c r="B107" s="13">
         <v>69</v>
       </c>
-      <c r="C107" s="16" t="s">
+      <c r="C107" s="9"/>
+      <c r="D107" s="16" t="s">
         <v>3882</v>
       </c>
-      <c r="D107" s="18">
+      <c r="E107" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="2:4">
+    <row r="108" spans="2:5">
       <c r="B108" s="13" t="s">
         <v>3883</v>
       </c>
-      <c r="C108" s="16"/>
-      <c r="D108" s="18">
+      <c r="C108" s="9"/>
+      <c r="D108" s="16"/>
+      <c r="E108" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="2:4">
+    <row r="109" spans="2:5">
       <c r="B109" s="13" t="s">
         <v>3884</v>
       </c>
-      <c r="C109" s="16"/>
-      <c r="D109" s="18">
+      <c r="C109" s="9"/>
+      <c r="D109" s="16"/>
+      <c r="E109" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="2:4">
+    <row r="110" spans="2:5">
       <c r="B110" s="13" t="s">
         <v>3885</v>
       </c>
-      <c r="C110" s="16"/>
-      <c r="D110" s="18">
+      <c r="C110" s="9"/>
+      <c r="D110" s="16"/>
+      <c r="E110" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="2:4">
+    <row r="111" spans="2:5">
       <c r="B111" s="13" t="s">
         <v>3886</v>
       </c>
-      <c r="C111" s="16"/>
-      <c r="D111" s="18">
+      <c r="C111" s="9"/>
+      <c r="D111" s="16"/>
+      <c r="E111" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="2:4">
+    <row r="112" spans="2:5">
       <c r="B112" s="13" t="s">
         <v>3887</v>
       </c>
-      <c r="C112" s="16"/>
-      <c r="D112" s="18">
+      <c r="C112" s="9"/>
+      <c r="D112" s="16"/>
+      <c r="E112" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:4">
+    <row r="113" spans="1:5">
       <c r="B113" s="13" t="s">
         <v>3810</v>
       </c>
-      <c r="C113" s="16"/>
-      <c r="D113" s="18">
+      <c r="C113" s="9"/>
+      <c r="D113" s="16"/>
+      <c r="E113" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:4">
+    <row r="114" spans="1:5">
       <c r="B114" s="13">
         <v>70</v>
       </c>
-      <c r="C114" s="16"/>
-      <c r="D114" s="18">
+      <c r="C114" s="9"/>
+      <c r="D114" s="16"/>
+      <c r="E114" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:4">
+    <row r="115" spans="1:5">
       <c r="B115" s="13">
         <v>71</v>
       </c>
-      <c r="C115" s="16"/>
-      <c r="D115" s="18">
+      <c r="C115" s="9"/>
+      <c r="D115" s="16"/>
+      <c r="E115" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:4">
+    <row r="116" spans="1:5">
       <c r="B116" s="13">
         <v>72</v>
       </c>
-      <c r="C116" s="16"/>
-      <c r="D116" s="18">
+      <c r="C116" s="9"/>
+      <c r="D116" s="16"/>
+      <c r="E116" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:4">
+    <row r="117" spans="1:5">
       <c r="B117" s="13">
         <v>73</v>
       </c>
-      <c r="C117" s="16"/>
-      <c r="D117" s="18">
+      <c r="C117" s="9"/>
+      <c r="D117" s="16"/>
+      <c r="E117" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:4">
+    <row r="118" spans="1:5">
       <c r="B118" s="13">
         <v>74</v>
       </c>
-      <c r="C118" s="16"/>
-      <c r="D118" s="18">
+      <c r="C118" s="9"/>
+      <c r="D118" s="16"/>
+      <c r="E118" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:4">
+    <row r="119" spans="1:5">
       <c r="B119" s="13">
         <v>75</v>
       </c>
-      <c r="C119" s="16"/>
-      <c r="D119" s="18">
+      <c r="C119" s="9"/>
+      <c r="D119" s="16"/>
+      <c r="E119" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:4">
+    <row r="120" spans="1:5">
       <c r="B120" s="13">
         <v>76</v>
       </c>
-      <c r="C120" s="16"/>
-      <c r="D120" s="18">
+      <c r="C120" s="9"/>
+      <c r="D120" s="16"/>
+      <c r="E120" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:4">
+    <row r="121" spans="1:5">
       <c r="B121" s="13">
         <v>77</v>
       </c>
-      <c r="C121" s="16"/>
-      <c r="D121" s="18">
+      <c r="C121" s="9"/>
+      <c r="D121" s="16"/>
+      <c r="E121" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:4">
+    <row r="122" spans="1:5">
       <c r="B122" s="13">
         <v>78</v>
       </c>
-      <c r="C122" s="16"/>
-      <c r="D122" s="18">
+      <c r="C122" s="9"/>
+      <c r="D122" s="16"/>
+      <c r="E122" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:4">
+    <row r="123" spans="1:5">
       <c r="B123" s="13">
         <v>79</v>
       </c>
-      <c r="C123" s="16"/>
-      <c r="D123" s="18">
+      <c r="C123" s="9"/>
+      <c r="D123" s="16"/>
+      <c r="E123" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="23" customHeight="1">
+    <row r="124" spans="1:5" ht="23" customHeight="1">
       <c r="A124" s="9" t="s">
-        <v>3888</v>
+        <v>4427</v>
       </c>
       <c r="B124" s="12" t="s">
         <v>3889</v>
       </c>
-      <c r="C124" s="15" t="s">
+      <c r="C124" s="9" t="s">
+        <v>3888</v>
+      </c>
+      <c r="D124" s="15" t="s">
         <v>3890</v>
       </c>
-      <c r="D124" s="18">
+      <c r="E124" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:4">
+    <row r="125" spans="1:5">
       <c r="B125" s="12" t="s">
         <v>3891</v>
       </c>
-      <c r="D125" s="18">
+      <c r="C125" s="9"/>
+      <c r="E125" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:4">
+    <row r="126" spans="1:5">
       <c r="B126" s="12" t="s">
         <v>3892</v>
       </c>
-      <c r="D126" s="18">
+      <c r="C126" s="9"/>
+      <c r="E126" s="18">
         <v>43</v>
       </c>
     </row>
-    <row r="127" spans="1:4">
+    <row r="127" spans="1:5">
       <c r="B127" s="12" t="s">
         <v>3893</v>
       </c>
-      <c r="D127" s="18">
+      <c r="C127" s="9"/>
+      <c r="E127" s="18">
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:4">
+    <row r="128" spans="1:5">
       <c r="B128" s="12" t="s">
         <v>3894</v>
       </c>
-      <c r="D128" s="18">
+      <c r="C128" s="9"/>
+      <c r="E128" s="18">
         <v>2</v>
       </c>
     </row>
-    <row r="129" spans="2:4">
+    <row r="129" spans="2:5">
       <c r="B129" s="12" t="s">
         <v>3824</v>
       </c>
-      <c r="D129" s="18" t="s">
+      <c r="E129" s="18" t="s">
         <v>1586</v>
       </c>
     </row>

</xml_diff>

<commit_message>
more fixes to get KLR running
</commit_message>
<xml_diff>
--- a/gemini8048/bin/87KLR951.xlsx
+++ b/gemini8048/bin/87KLR951.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mike/coding_projects/944/DME_sim/gemini8048/bin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EFA0F05-AC71-694D-9A54-DEA9E9F0CFF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD8A813D-1549-B249-90FC-10D2045F3EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37360" yWindow="8740" windowWidth="47100" windowHeight="24480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3920" yWindow="18100" windowWidth="47100" windowHeight="24480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ASM" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8162" uniqueCount="4429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8163" uniqueCount="4429">
   <si>
     <t>https://junctionbyte.com/8051-microcontroller-special-function-registers/</t>
   </si>
@@ -13437,7 +13437,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -13497,6 +13497,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -13841,7 +13844,7 @@
     <col min="4" max="4" width="14.5" customWidth="1"/>
     <col min="5" max="5" width="25.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="26.6640625" customWidth="1"/>
-    <col min="7" max="7" width="80.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="59" customWidth="1"/>
     <col min="8" max="8" width="61.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="80.6640625" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="72" customWidth="1"/>
@@ -26813,6 +26816,9 @@
     <row r="701" spans="1:34">
       <c r="A701" t="s">
         <v>2166</v>
+      </c>
+      <c r="B701" s="27" t="s">
+        <v>117</v>
       </c>
       <c r="C701" s="1" t="s">
         <v>2167</v>

</xml_diff>

<commit_message>
1st submit for verialtor compatible code
</commit_message>
<xml_diff>
--- a/gemini8048/bin/87KLR951.xlsx
+++ b/gemini8048/bin/87KLR951.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mike/coding_projects/944/DME_sim/gemini8048/bin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C2AEDB-3118-744F-91F3-05DB9B46F31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1C6CC1-E034-104A-A412-2F5E561912E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12760" yWindow="11380" windowWidth="39200" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12760" yWindow="11380" windowWidth="48760" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ASM" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8144" uniqueCount="4410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8147" uniqueCount="4413">
   <si>
     <t>https://junctionbyte.com/8051-microcontroller-special-function-registers/</t>
   </si>
@@ -13264,9 +13264,6 @@
     <t>knock_thresh_coeef</t>
   </si>
   <si>
-    <t>// get value from map addr = 925 (2AH)</t>
-  </si>
-  <si>
     <t>// r2 gets 2eH</t>
   </si>
   <si>
@@ -13277,6 +13274,18 @@
   </si>
   <si>
     <t>// store 7f into mem[2a]</t>
+  </si>
+  <si>
+    <t>// 1st pass: get value from map addr = 925 (2AH), 2nd pass from 92eh (2bh)</t>
+  </si>
+  <si>
+    <t>eventually exits loop at map addr 991</t>
+  </si>
+  <si>
+    <t>//get byte from addr 9B1 (e3H)</t>
+  </si>
+  <si>
+    <t>data at end of map lookup gets stored here (code addr = 923)</t>
   </si>
 </sst>
 </file>
@@ -26756,7 +26765,7 @@
         <v>2153</v>
       </c>
     </row>
-    <row r="705" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="705" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A705" t="s">
         <v>2154</v>
       </c>
@@ -26773,7 +26782,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="706" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="706" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A706" t="s">
         <v>2155</v>
       </c>
@@ -26790,7 +26799,7 @@
         <v>1591</v>
       </c>
     </row>
-    <row r="707" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="707" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A707" t="s">
         <v>2156</v>
       </c>
@@ -26807,7 +26816,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="708" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="708" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A708" t="s">
         <v>2157</v>
       </c>
@@ -26824,7 +26833,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="709" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="709" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A709" t="s">
         <v>2158</v>
       </c>
@@ -26841,7 +26850,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="710" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="710" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A710" t="s">
         <v>2159</v>
       </c>
@@ -26858,7 +26867,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="711" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="711" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A711" t="s">
         <v>2160</v>
       </c>
@@ -26875,7 +26884,7 @@
         <v>2163</v>
       </c>
     </row>
-    <row r="712" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="712" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A712" t="s">
         <v>2164</v>
       </c>
@@ -26895,7 +26904,7 @@
         <v>2165</v>
       </c>
     </row>
-    <row r="713" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="713" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A713" t="s">
         <v>2166</v>
       </c>
@@ -26912,10 +26921,13 @@
         <v>630</v>
       </c>
       <c r="G713" s="1" t="s">
-        <v>4405</v>
-      </c>
-    </row>
-    <row r="714" spans="1:7" x14ac:dyDescent="0.2">
+        <v>4409</v>
+      </c>
+      <c r="H713" t="s">
+        <v>4410</v>
+      </c>
+    </row>
+    <row r="714" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A714" t="s">
         <v>2167</v>
       </c>
@@ -26932,7 +26944,7 @@
         <v>2170</v>
       </c>
     </row>
-    <row r="715" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="715" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A715" t="s">
         <v>2171</v>
       </c>
@@ -26949,7 +26961,7 @@
         <v>1623</v>
       </c>
     </row>
-    <row r="716" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="716" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A716" t="s">
         <v>2172</v>
       </c>
@@ -26966,7 +26978,7 @@
         <v>2165</v>
       </c>
     </row>
-    <row r="717" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="717" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A717" t="s">
         <v>2173</v>
       </c>
@@ -26984,7 +26996,7 @@
       </c>
       <c r="G717" s="1"/>
     </row>
-    <row r="718" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="718" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A718" t="s">
         <v>2177</v>
       </c>
@@ -27001,10 +27013,10 @@
         <v>149</v>
       </c>
       <c r="G718" s="1" t="s">
-        <v>4406</v>
-      </c>
-    </row>
-    <row r="719" spans="1:7" x14ac:dyDescent="0.2">
+        <v>4405</v>
+      </c>
+    </row>
+    <row r="719" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A719" t="s">
         <v>2178</v>
       </c>
@@ -27021,10 +27033,10 @@
         <v>2181</v>
       </c>
       <c r="G719" s="1" t="s">
-        <v>4407</v>
-      </c>
-    </row>
-    <row r="720" spans="1:7" x14ac:dyDescent="0.2">
+        <v>4406</v>
+      </c>
+    </row>
+    <row r="720" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A720" t="s">
         <v>2182</v>
       </c>
@@ -27041,7 +27053,7 @@
         <v>630</v>
       </c>
       <c r="G720" s="1" t="s">
-        <v>4408</v>
+        <v>4407</v>
       </c>
     </row>
     <row r="721" spans="1:8" x14ac:dyDescent="0.2">
@@ -27061,7 +27073,7 @@
         <v>387</v>
       </c>
       <c r="G721" s="1" t="s">
-        <v>4409</v>
+        <v>4408</v>
       </c>
     </row>
     <row r="722" spans="1:8" x14ac:dyDescent="0.2">
@@ -27187,6 +27199,9 @@
       </c>
       <c r="F728" t="s">
         <v>630</v>
+      </c>
+      <c r="G728" s="1" t="s">
+        <v>4411</v>
       </c>
     </row>
     <row r="729" spans="1:8" x14ac:dyDescent="0.2">
@@ -41393,12 +41408,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:5" ht="23" x14ac:dyDescent="0.3">
       <c r="B109" s="13" t="s">
         <v>3860</v>
       </c>
       <c r="C109" s="9"/>
-      <c r="D109" s="16"/>
+      <c r="D109" s="16" t="s">
+        <v>4412</v>
+      </c>
       <c r="E109" s="18">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Verilator fixes: i8051_dashboard_tb ifndef guards, FST output, validate unimplemented opcode check, run script cleanup
</commit_message>
<xml_diff>
--- a/gemini8048/bin/87KLR951.xlsx
+++ b/gemini8048/bin/87KLR951.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mike/coding_projects/944/DME_sim/gemini8048/bin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1C6CC1-E034-104A-A412-2F5E561912E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72EBECBC-8B97-944C-A509-9307ABBADC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12760" yWindow="11380" windowWidth="48760" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16140" yWindow="12620" windowWidth="48760" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ASM" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8147" uniqueCount="4413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8149" uniqueCount="4416">
   <si>
     <t>https://junctionbyte.com/8051-microcontroller-special-function-registers/</t>
   </si>
@@ -13286,6 +13286,15 @@
   </si>
   <si>
     <t>data at end of map lookup gets stored here (code addr = 923)</t>
+  </si>
+  <si>
+    <t>//wrong call - goes to C80 not 480</t>
+  </si>
+  <si>
+    <t>labelb80:</t>
+  </si>
+  <si>
+    <t>label0b80</t>
   </si>
 </sst>
 </file>
@@ -13791,7 +13800,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="9.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="14.5" customWidth="1"/>
     <col min="5" max="5" width="25.33203125" style="1" customWidth="1"/>
@@ -29058,6 +29067,9 @@
       <c r="F829" t="s">
         <v>2434</v>
       </c>
+      <c r="G829" s="1" t="s">
+        <v>4413</v>
+      </c>
     </row>
     <row r="830" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A830" t="s">
@@ -29232,7 +29244,7 @@
         <v>323</v>
       </c>
       <c r="E839" s="1" t="s">
-        <v>2459</v>
+        <v>4415</v>
       </c>
       <c r="F839" t="s">
         <v>2460</v>
@@ -29403,6 +29415,9 @@
     <row r="849" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A849" t="s">
         <v>2481</v>
+      </c>
+      <c r="B849" t="s">
+        <v>4414</v>
       </c>
       <c r="C849" s="1" t="s">
         <v>130</v>

</xml_diff>

<commit_message>
Add o2_baseline test, O2 sensor validation, and comparator improvements
- compare_sim_logs.py: 16-bit hb/lb field merging, flags(21)/(23)/(25)
  split, per-test and global field ignore lists, consecutive-mismatch
  filtering, --plot/--verbose/--field/--list-fields options
- run_dashboard_tests.sh / v_run_dashboard_tests.sh: new o2_baseline test
- validate_dash_log.py: O2 sensor status check (R3e + B26)
- compare_all_logs.sh: add o2_baseline to test lists
- run_all.sh: auto-generate compare_sim_logs.py detail/plots for DIFF tests
- i8051_dashboard_tb.v, vcd.v, dme_analog_O2_recovery_test.asc,
  disassemble2.xlsx, 87KLR951.xlsx: [add a short note on what changed here]
</commit_message>
<xml_diff>
--- a/gemini8048/bin/87KLR951.xlsx
+++ b/gemini8048/bin/87KLR951.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mike/coding_projects/944/DME_sim/gemini8048/bin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72EBECBC-8B97-944C-A509-9307ABBADC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF0E645-6EEC-734C-B36B-605E80B71C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16140" yWindow="12620" windowWidth="48760" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="49000" yWindow="17460" windowWidth="48760" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ASM" sheetId="1" r:id="rId1"/>

</xml_diff>